<commit_message>
Add marc.png image to avocattest8 site
</commit_message>
<xml_diff>
--- a/base de donnees num.xlsx
+++ b/base de donnees num.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harri\OneDrive\Bureau\Site drop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB79379-4D82-4161-9D3D-C01DF1832D57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FA44F4-E442-4EAC-AB25-D484FA0A8FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{31BF64A7-4869-4DE3-9947-0E770714EAC3}"/>
+    <workbookView xWindow="3750" yWindow="2415" windowWidth="21600" windowHeight="11295" xr2:uid="{31BF64A7-4869-4DE3-9947-0E770714EAC3}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>TOULON</t>
   </si>
@@ -157,13 +157,25 @@
   </si>
   <si>
     <t>06.19.51.05.53 Sarl Lb Auto Racing</t>
+  </si>
+  <si>
+    <t>06 52 30 33 89 Hone Space</t>
+  </si>
+  <si>
+    <t>06.66.01.12.94 estelle collette</t>
+  </si>
+  <si>
+    <t>06.85.40.77.39 Marlin Julien</t>
+  </si>
+  <si>
+    <t>06.46.56.16.11 Oreggia Marc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,8 +189,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -218,6 +236,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -249,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -263,9 +293,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -276,6 +303,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -627,11 +666,11 @@
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D1" s="3"/>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>31</v>
       </c>
     </row>
@@ -641,150 +680,164 @@
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="10" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>6</v>
       </c>
+      <c r="C14" s="12" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>7</v>
       </c>
+      <c r="C15" s="11" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>8</v>
       </c>
+      <c r="C16" s="11" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="6" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>